<commit_message>
feat: adiciona sistema de ressarcimento de bots
- Implementa cálculo de ressarcimentos para contas suspeitas
- Adiciona conversão automática de moedas por liga
- Implementa sistema de acumulação para valores abaixo do mínimo
- Adiciona exportação em múltiplos formatos (String, CSV, Excel)
- Suporta upload de acumulados anteriores para continuidade entre semanas
- Utiliza session state para persistência de resultados
- Pronto para deploy no Streamlit Cloud
</commit_message>
<xml_diff>
--- a/ip_lookup/output/ip_geoloc.xlsx
+++ b/ip_lookup/output/ip_geoloc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://supremagroup-my.sharepoint.com/personal/douglas_ferreira_suprema_group/Documents/Suprema/DataForge_PKR/DataForge_PKR/ip_lookup/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD3F0571217D8291159D6A8736CA1FF66" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CB6CAF4-A172-42D5-8ACA-4D6FDEAFE59A}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_766951B6D340D906E3DA3911595ED87656CD9570" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A78376F1-A1FB-4727-A634-8FD17EC73AFB}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="1095" windowWidth="34890" windowHeight="20505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="94">
   <si>
     <t>ip_consultado</t>
   </si>
@@ -67,7 +67,7 @@
     <t>hospedagem</t>
   </si>
   <si>
-    <t>149.19.165.121</t>
+    <t>148.222.206.228</t>
   </si>
   <si>
     <t>success</t>
@@ -94,46 +94,214 @@
     <t>AS14593 Space Exploration Technologies Corporation</t>
   </si>
   <si>
-    <t>177.132.149.85</t>
-  </si>
-  <si>
-    <t>Paraná</t>
-  </si>
-  <si>
-    <t>Toledo</t>
-  </si>
-  <si>
-    <t>85900</t>
-  </si>
-  <si>
-    <t>TELEFÔNICA BRASIL S.A</t>
-  </si>
-  <si>
-    <t>Global Village Telecom</t>
-  </si>
-  <si>
-    <t>AS18881 TELEFÔNICA BRASIL S.A</t>
-  </si>
-  <si>
-    <t>177.156.17.126</t>
-  </si>
-  <si>
-    <t>128.201.1.34</t>
-  </si>
-  <si>
-    <t>Minas Gerais</t>
-  </si>
-  <si>
-    <t>Ipatinga</t>
-  </si>
-  <si>
-    <t>35160</t>
-  </si>
-  <si>
-    <t>Vero S.A</t>
-  </si>
-  <si>
-    <t>AS263405 VERO S.A</t>
+    <t>177.174.192.205</t>
+  </si>
+  <si>
+    <t>Rio Grande do Sul</t>
+  </si>
+  <si>
+    <t>Porto Alegre</t>
+  </si>
+  <si>
+    <t>90000</t>
+  </si>
+  <si>
+    <t>Vivo</t>
+  </si>
+  <si>
+    <t>TELEF�NICA BRASIL S.A</t>
+  </si>
+  <si>
+    <t>AS26599 TELEFÔNICA BRASIL S.A</t>
+  </si>
+  <si>
+    <t>177.174.192.252</t>
+  </si>
+  <si>
+    <t>177.174.193.27</t>
+  </si>
+  <si>
+    <t>177.174.193.64</t>
+  </si>
+  <si>
+    <t>177.174.194.103</t>
+  </si>
+  <si>
+    <t>177.174.194.252</t>
+  </si>
+  <si>
+    <t>177.174.195.5</t>
+  </si>
+  <si>
+    <t>177.174.195.72</t>
+  </si>
+  <si>
+    <t>177.174.196.235</t>
+  </si>
+  <si>
+    <t>177.174.197.108</t>
+  </si>
+  <si>
+    <t>177.174.197.45</t>
+  </si>
+  <si>
+    <t>177.174.198.189</t>
+  </si>
+  <si>
+    <t>177.174.198.195</t>
+  </si>
+  <si>
+    <t>177.174.198.93</t>
+  </si>
+  <si>
+    <t>177.174.199.1</t>
+  </si>
+  <si>
+    <t>177.174.199.139</t>
+  </si>
+  <si>
+    <t>177.174.199.37</t>
+  </si>
+  <si>
+    <t>177.174.200.192</t>
+  </si>
+  <si>
+    <t>177.174.200.245</t>
+  </si>
+  <si>
+    <t>177.174.200.80</t>
+  </si>
+  <si>
+    <t>177.174.201.237</t>
+  </si>
+  <si>
+    <t>177.174.201.84</t>
+  </si>
+  <si>
+    <t>177.174.202.167</t>
+  </si>
+  <si>
+    <t>177.174.202.187</t>
+  </si>
+  <si>
+    <t>177.174.202.189</t>
+  </si>
+  <si>
+    <t>177.174.202.72</t>
+  </si>
+  <si>
+    <t>177.174.203.109</t>
+  </si>
+  <si>
+    <t>177.174.204.187</t>
+  </si>
+  <si>
+    <t>177.174.204.196</t>
+  </si>
+  <si>
+    <t>177.174.205.105</t>
+  </si>
+  <si>
+    <t>177.174.205.61</t>
+  </si>
+  <si>
+    <t>177.174.206.141</t>
+  </si>
+  <si>
+    <t>177.174.206.175</t>
+  </si>
+  <si>
+    <t>177.174.206.50</t>
+  </si>
+  <si>
+    <t>177.174.206.51</t>
+  </si>
+  <si>
+    <t>177.174.207.104</t>
+  </si>
+  <si>
+    <t>177.174.244.119</t>
+  </si>
+  <si>
+    <t>Santa Catarina</t>
+  </si>
+  <si>
+    <t>Balneário Camboriú</t>
+  </si>
+  <si>
+    <t>88330</t>
+  </si>
+  <si>
+    <t>179.124.182.128</t>
+  </si>
+  <si>
+    <t>Santa Cruz do Sul</t>
+  </si>
+  <si>
+    <t>96800</t>
+  </si>
+  <si>
+    <t>Roberto Keller - ME</t>
+  </si>
+  <si>
+    <t>AS61914 Roberto Keller - ME</t>
+  </si>
+  <si>
+    <t>179.124.182.188</t>
+  </si>
+  <si>
+    <t>179.124.183.160</t>
+  </si>
+  <si>
+    <t>Traudi Ines Sehnem</t>
+  </si>
+  <si>
+    <t>179.151.164.96</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Nilópolis</t>
+  </si>
+  <si>
+    <t>28000-000</t>
+  </si>
+  <si>
+    <t>187.45.101.159</t>
+  </si>
+  <si>
+    <t>Mhnet Telecom</t>
+  </si>
+  <si>
+    <t>AS28146 MHNET TELECOM</t>
+  </si>
+  <si>
+    <t>187.66.39.84</t>
+  </si>
+  <si>
+    <t>96810</t>
+  </si>
+  <si>
+    <t>Claro NXT Telecomunicacoes Ltda</t>
+  </si>
+  <si>
+    <t>NET Serviços de Comunicação S.A.</t>
+  </si>
+  <si>
+    <t>AS28573 Claro NXT Telecomunicacoes Ltda</t>
+  </si>
+  <si>
+    <t>45.175.25.36</t>
+  </si>
+  <si>
+    <t>96840</t>
+  </si>
+  <si>
+    <t>RASÃO SYGANET TELECOMUNICAÇÕES LTDA</t>
+  </si>
+  <si>
+    <t>AS268879 RASÃO SYGANET TELECOMUNICAÇÕES LTDA</t>
   </si>
 </sst>
 </file>
@@ -497,8 +665,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5703125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="40.28515625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="49.28515625" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5703125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="6.140625" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="12.42578125" hidden="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -620,10 +805,10 @@
         <v>30</v>
       </c>
       <c r="L3">
-        <v>-24.733699999999999</v>
+        <v>-30.1188</v>
       </c>
       <c r="M3">
-        <v>-53.8202</v>
+        <v>-51.167999999999999</v>
       </c>
       <c r="N3" t="b">
         <v>0</v>
@@ -664,10 +849,10 @@
         <v>30</v>
       </c>
       <c r="L4">
-        <v>-24.733699999999999</v>
+        <v>-30.1188</v>
       </c>
       <c r="M4">
-        <v>-53.8202</v>
+        <v>-51.167999999999999</v>
       </c>
       <c r="N4" t="b">
         <v>0</v>
@@ -687,71 +872,1838 @@
         <v>17</v>
       </c>
       <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L5">
+        <v>-30.1188</v>
+      </c>
+      <c r="M5">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K5" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5">
-        <v>-19.438600000000001</v>
-      </c>
-      <c r="M5">
-        <v>-42.606000000000002</v>
-      </c>
-      <c r="N5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" t="b">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L6">
+        <v>-30.1188</v>
+      </c>
+      <c r="M6">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>8</v>
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" t="s">
+        <v>30</v>
+      </c>
+      <c r="L7">
+        <v>-30.1188</v>
+      </c>
+      <c r="M7">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8">
+        <v>-30.1188</v>
+      </c>
+      <c r="M8">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" t="s">
+        <v>29</v>
+      </c>
+      <c r="K9" t="s">
+        <v>30</v>
+      </c>
+      <c r="L9">
+        <v>-30.1188</v>
+      </c>
+      <c r="M9">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" t="s">
+        <v>30</v>
+      </c>
+      <c r="L10">
+        <v>-30.1188</v>
+      </c>
+      <c r="M10">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" t="s">
+        <v>30</v>
+      </c>
+      <c r="L11">
+        <v>-30.1188</v>
+      </c>
+      <c r="M11">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" t="s">
+        <v>29</v>
+      </c>
+      <c r="K12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L12">
+        <v>-30.1188</v>
+      </c>
+      <c r="M12">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L13">
+        <v>-30.1188</v>
+      </c>
+      <c r="M13">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N13" t="b">
+        <v>0</v>
+      </c>
+      <c r="O13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" t="s">
+        <v>30</v>
+      </c>
+      <c r="L14">
+        <v>-30.1188</v>
+      </c>
+      <c r="M14">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" t="s">
+        <v>29</v>
+      </c>
+      <c r="K15" t="s">
+        <v>30</v>
+      </c>
+      <c r="L15">
+        <v>-30.1188</v>
+      </c>
+      <c r="M15">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" t="s">
+        <v>29</v>
+      </c>
+      <c r="K16" t="s">
+        <v>30</v>
+      </c>
+      <c r="L16">
+        <v>-30.1188</v>
+      </c>
+      <c r="M16">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" t="s">
+        <v>29</v>
+      </c>
+      <c r="K17" t="s">
+        <v>30</v>
+      </c>
+      <c r="L17">
+        <v>-30.1188</v>
+      </c>
+      <c r="M17">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" t="s">
+        <v>29</v>
+      </c>
+      <c r="K18" t="s">
+        <v>30</v>
+      </c>
+      <c r="L18">
+        <v>-30.1188</v>
+      </c>
+      <c r="M18">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J19" t="s">
+        <v>29</v>
+      </c>
+      <c r="K19" t="s">
+        <v>30</v>
+      </c>
+      <c r="L19">
+        <v>-30.1188</v>
+      </c>
+      <c r="M19">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" t="s">
+        <v>20</v>
+      </c>
+      <c r="I20" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" t="s">
+        <v>29</v>
+      </c>
+      <c r="K20" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20">
+        <v>-30.1188</v>
+      </c>
+      <c r="M20">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+      <c r="O20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" t="s">
+        <v>28</v>
+      </c>
+      <c r="J21" t="s">
+        <v>29</v>
+      </c>
+      <c r="K21" t="s">
+        <v>30</v>
+      </c>
+      <c r="L21">
+        <v>-30.1188</v>
+      </c>
+      <c r="M21">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N21" t="b">
+        <v>0</v>
+      </c>
+      <c r="O21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" t="s">
+        <v>20</v>
+      </c>
+      <c r="I22" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" t="s">
+        <v>29</v>
+      </c>
+      <c r="K22" t="s">
+        <v>30</v>
+      </c>
+      <c r="L22">
+        <v>-30.1188</v>
+      </c>
+      <c r="M22">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" t="s">
+        <v>27</v>
+      </c>
+      <c r="H23" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" t="s">
+        <v>28</v>
+      </c>
+      <c r="J23" t="s">
+        <v>29</v>
+      </c>
+      <c r="K23" t="s">
+        <v>30</v>
+      </c>
+      <c r="L23">
+        <v>-30.1188</v>
+      </c>
+      <c r="M23">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" t="s">
+        <v>20</v>
+      </c>
+      <c r="I24" t="s">
+        <v>28</v>
+      </c>
+      <c r="J24" t="s">
+        <v>29</v>
+      </c>
+      <c r="K24" t="s">
+        <v>30</v>
+      </c>
+      <c r="L24">
+        <v>-30.1188</v>
+      </c>
+      <c r="M24">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" t="s">
+        <v>27</v>
+      </c>
+      <c r="H25" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" t="s">
+        <v>29</v>
+      </c>
+      <c r="K25" t="s">
+        <v>30</v>
+      </c>
+      <c r="L25">
+        <v>-30.1188</v>
+      </c>
+      <c r="M25">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" t="s">
+        <v>25</v>
+      </c>
+      <c r="F26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" t="s">
+        <v>27</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" t="s">
+        <v>29</v>
+      </c>
+      <c r="K26" t="s">
+        <v>30</v>
+      </c>
+      <c r="L26">
+        <v>-30.1188</v>
+      </c>
+      <c r="M26">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+      <c r="I27" t="s">
+        <v>28</v>
+      </c>
+      <c r="J27" t="s">
+        <v>29</v>
+      </c>
+      <c r="K27" t="s">
+        <v>30</v>
+      </c>
+      <c r="L27">
+        <v>-30.1188</v>
+      </c>
+      <c r="M27">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I28" t="s">
+        <v>28</v>
+      </c>
+      <c r="J28" t="s">
+        <v>29</v>
+      </c>
+      <c r="K28" t="s">
+        <v>30</v>
+      </c>
+      <c r="L28">
+        <v>-30.1188</v>
+      </c>
+      <c r="M28">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N28" t="b">
+        <v>0</v>
+      </c>
+      <c r="O28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" t="s">
+        <v>28</v>
+      </c>
+      <c r="J29" t="s">
+        <v>29</v>
+      </c>
+      <c r="K29" t="s">
+        <v>30</v>
+      </c>
+      <c r="L29">
+        <v>-30.1188</v>
+      </c>
+      <c r="M29">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N29" t="b">
+        <v>0</v>
+      </c>
+      <c r="O29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I30" t="s">
+        <v>28</v>
+      </c>
+      <c r="J30" t="s">
+        <v>29</v>
+      </c>
+      <c r="K30" t="s">
+        <v>30</v>
+      </c>
+      <c r="L30">
+        <v>-30.1188</v>
+      </c>
+      <c r="M30">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N30" t="b">
+        <v>0</v>
+      </c>
+      <c r="O30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" t="s">
+        <v>27</v>
+      </c>
+      <c r="H31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I31" t="s">
+        <v>28</v>
+      </c>
+      <c r="J31" t="s">
+        <v>29</v>
+      </c>
+      <c r="K31" t="s">
+        <v>30</v>
+      </c>
+      <c r="L31">
+        <v>-30.1188</v>
+      </c>
+      <c r="M31">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N31" t="b">
+        <v>0</v>
+      </c>
+      <c r="O31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" t="s">
+        <v>26</v>
+      </c>
+      <c r="G32" t="s">
+        <v>27</v>
+      </c>
+      <c r="H32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" t="s">
+        <v>28</v>
+      </c>
+      <c r="J32" t="s">
+        <v>29</v>
+      </c>
+      <c r="K32" t="s">
+        <v>30</v>
+      </c>
+      <c r="L32">
+        <v>-30.1188</v>
+      </c>
+      <c r="M32">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" t="s">
+        <v>29</v>
+      </c>
+      <c r="K33" t="s">
+        <v>30</v>
+      </c>
+      <c r="L33">
+        <v>-30.1188</v>
+      </c>
+      <c r="M33">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" t="s">
+        <v>27</v>
+      </c>
+      <c r="H34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" t="s">
+        <v>28</v>
+      </c>
+      <c r="J34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K34" t="s">
+        <v>30</v>
+      </c>
+      <c r="L34">
+        <v>-30.1188</v>
+      </c>
+      <c r="M34">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N34" t="b">
+        <v>0</v>
+      </c>
+      <c r="O34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" t="s">
+        <v>17</v>
+      </c>
+      <c r="E35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" t="s">
+        <v>27</v>
+      </c>
+      <c r="H35" t="s">
+        <v>20</v>
+      </c>
+      <c r="I35" t="s">
+        <v>28</v>
+      </c>
+      <c r="J35" t="s">
+        <v>29</v>
+      </c>
+      <c r="K35" t="s">
+        <v>30</v>
+      </c>
+      <c r="L35">
+        <v>-30.1188</v>
+      </c>
+      <c r="M35">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N35" t="b">
+        <v>0</v>
+      </c>
+      <c r="O35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" t="s">
+        <v>26</v>
+      </c>
+      <c r="G36" t="s">
+        <v>27</v>
+      </c>
+      <c r="H36" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" t="s">
+        <v>28</v>
+      </c>
+      <c r="J36" t="s">
+        <v>29</v>
+      </c>
+      <c r="K36" t="s">
+        <v>30</v>
+      </c>
+      <c r="L36">
+        <v>-30.1188</v>
+      </c>
+      <c r="M36">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N36" t="b">
+        <v>0</v>
+      </c>
+      <c r="O36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" t="s">
+        <v>17</v>
+      </c>
+      <c r="E37" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" t="s">
+        <v>27</v>
+      </c>
+      <c r="H37" t="s">
+        <v>20</v>
+      </c>
+      <c r="I37" t="s">
+        <v>28</v>
+      </c>
+      <c r="J37" t="s">
+        <v>29</v>
+      </c>
+      <c r="K37" t="s">
+        <v>30</v>
+      </c>
+      <c r="L37">
+        <v>-30.1188</v>
+      </c>
+      <c r="M37">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N37" t="b">
+        <v>0</v>
+      </c>
+      <c r="O37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+      <c r="D38" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" t="s">
+        <v>26</v>
+      </c>
+      <c r="G38" t="s">
+        <v>27</v>
+      </c>
+      <c r="H38" t="s">
+        <v>20</v>
+      </c>
+      <c r="I38" t="s">
+        <v>28</v>
+      </c>
+      <c r="J38" t="s">
+        <v>29</v>
+      </c>
+      <c r="K38" t="s">
+        <v>30</v>
+      </c>
+      <c r="L38">
+        <v>-30.1188</v>
+      </c>
+      <c r="M38">
+        <v>-51.167999999999999</v>
+      </c>
+      <c r="N38" t="b">
+        <v>0</v>
+      </c>
+      <c r="O38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" t="s">
+        <v>67</v>
+      </c>
+      <c r="F39" t="s">
+        <v>68</v>
+      </c>
+      <c r="G39" t="s">
+        <v>69</v>
+      </c>
+      <c r="H39" t="s">
+        <v>20</v>
+      </c>
+      <c r="I39" t="s">
+        <v>28</v>
+      </c>
+      <c r="J39" t="s">
+        <v>29</v>
+      </c>
+      <c r="K39" t="s">
+        <v>30</v>
+      </c>
+      <c r="L39">
+        <v>-26.998100000000001</v>
+      </c>
+      <c r="M39">
+        <v>-48.618699999999997</v>
+      </c>
+      <c r="N39" t="b">
+        <v>0</v>
+      </c>
+      <c r="O39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" t="s">
+        <v>17</v>
+      </c>
+      <c r="E40" t="s">
+        <v>25</v>
+      </c>
+      <c r="F40" t="s">
+        <v>71</v>
+      </c>
+      <c r="G40" t="s">
+        <v>72</v>
+      </c>
+      <c r="H40" t="s">
+        <v>20</v>
+      </c>
+      <c r="I40" t="s">
+        <v>73</v>
+      </c>
+      <c r="J40" t="s">
+        <v>73</v>
+      </c>
+      <c r="K40" t="s">
+        <v>74</v>
+      </c>
+      <c r="L40">
+        <v>-29.615300000000001</v>
+      </c>
+      <c r="M40">
+        <v>-52.411000000000001</v>
+      </c>
+      <c r="N40" t="b">
+        <v>0</v>
+      </c>
+      <c r="O40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D41" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" t="s">
+        <v>25</v>
+      </c>
+      <c r="F41" t="s">
+        <v>71</v>
+      </c>
+      <c r="G41" t="s">
+        <v>72</v>
+      </c>
+      <c r="H41" t="s">
+        <v>20</v>
+      </c>
+      <c r="I41" t="s">
+        <v>73</v>
+      </c>
+      <c r="J41" t="s">
+        <v>73</v>
+      </c>
+      <c r="K41" t="s">
+        <v>74</v>
+      </c>
+      <c r="L41">
+        <v>-29.615300000000001</v>
+      </c>
+      <c r="M41">
+        <v>-52.411000000000001</v>
+      </c>
+      <c r="N41" t="b">
+        <v>0</v>
+      </c>
+      <c r="O41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42" t="s">
+        <v>71</v>
+      </c>
+      <c r="G42" t="s">
+        <v>72</v>
+      </c>
+      <c r="H42" t="s">
+        <v>20</v>
+      </c>
+      <c r="I42" t="s">
+        <v>73</v>
+      </c>
+      <c r="J42" t="s">
+        <v>77</v>
+      </c>
+      <c r="K42" t="s">
+        <v>74</v>
+      </c>
+      <c r="L42">
+        <v>-29.615300000000001</v>
+      </c>
+      <c r="M42">
+        <v>-52.411000000000001</v>
+      </c>
+      <c r="N42" t="b">
+        <v>0</v>
+      </c>
+      <c r="O42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" t="s">
+        <v>17</v>
+      </c>
+      <c r="E43" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" t="s">
+        <v>80</v>
+      </c>
+      <c r="G43" t="s">
+        <v>81</v>
+      </c>
+      <c r="H43" t="s">
+        <v>20</v>
+      </c>
+      <c r="I43" t="s">
+        <v>28</v>
+      </c>
+      <c r="J43" t="s">
+        <v>29</v>
+      </c>
+      <c r="K43" t="s">
+        <v>30</v>
+      </c>
+      <c r="L43">
+        <v>-22.807500000000001</v>
+      </c>
+      <c r="M43">
+        <v>-43.413899999999998</v>
+      </c>
+      <c r="N43" t="b">
+        <v>0</v>
+      </c>
+      <c r="O43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" t="s">
+        <v>17</v>
+      </c>
+      <c r="E44" t="s">
+        <v>25</v>
+      </c>
+      <c r="F44" t="s">
+        <v>71</v>
+      </c>
+      <c r="H44" t="s">
+        <v>20</v>
+      </c>
+      <c r="I44" t="s">
+        <v>83</v>
+      </c>
+      <c r="J44" t="s">
+        <v>83</v>
+      </c>
+      <c r="K44" t="s">
+        <v>84</v>
+      </c>
+      <c r="L44">
+        <v>-29.717500000000001</v>
+      </c>
+      <c r="M44">
+        <v>-52.425800000000002</v>
+      </c>
+      <c r="N44" t="b">
+        <v>0</v>
+      </c>
+      <c r="O44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" t="s">
+        <v>16</v>
+      </c>
+      <c r="D45" t="s">
+        <v>17</v>
+      </c>
+      <c r="E45" t="s">
+        <v>25</v>
+      </c>
+      <c r="F45" t="s">
+        <v>71</v>
+      </c>
+      <c r="G45" t="s">
+        <v>86</v>
+      </c>
+      <c r="H45" t="s">
+        <v>20</v>
+      </c>
+      <c r="I45" t="s">
+        <v>87</v>
+      </c>
+      <c r="J45" t="s">
+        <v>88</v>
+      </c>
+      <c r="K45" t="s">
+        <v>89</v>
+      </c>
+      <c r="L45">
+        <v>-29.718</v>
+      </c>
+      <c r="M45">
+        <v>-52.426600000000001</v>
+      </c>
+      <c r="N45" t="b">
+        <v>0</v>
+      </c>
+      <c r="O45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" t="s">
+        <v>17</v>
+      </c>
+      <c r="E46" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46" t="s">
+        <v>71</v>
+      </c>
+      <c r="G46" t="s">
+        <v>91</v>
+      </c>
+      <c r="H46" t="s">
+        <v>20</v>
+      </c>
+      <c r="I46" t="s">
+        <v>92</v>
+      </c>
+      <c r="J46" t="s">
+        <v>92</v>
+      </c>
+      <c r="K46" t="s">
+        <v>93</v>
+      </c>
+      <c r="L46">
+        <v>-29.718</v>
+      </c>
+      <c r="M46">
+        <v>-52.426600000000001</v>
+      </c>
+      <c r="N46" t="b">
+        <v>0</v>
+      </c>
+      <c r="O46" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>